<commit_message>
Libretto Marco: Fasi 1, 2 e 3
Aggiunte le tre voci scritte insieme a Manuel, datate 30/09/2026, con
una stima di un'ora ciascuna.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/libretti/marco-buffa.xlsx
+++ b/docs/libretti/marco-buffa.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\bulla\AppData\Local\Temp\claude\C--Users-bulla-Documents-Ing-software-v1\c32cf868-ae9e-4ff3-a799-856eab5b1d43\scratchpad\out\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\bulla\Documents\Ing-software-v1\docs\libretti\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{A5FD70AE-A7E4-4D51-ACF1-C96C71BB2D75}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{18DB9327-8DE3-46DC-9CA1-1444C9B38741}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" xr2:uid="{69E2A5B4-4109-48EA-BF49-3C21B144A51A}"/>
   </bookViews>
@@ -43,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="28">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="39" uniqueCount="37">
   <si>
     <t>Libretto delle attività</t>
   </si>
@@ -127,6 +127,33 @@
   </si>
   <si>
     <t>Se 'Fuori dalle settimane elencate' non è zero, ci sono voci con una data oltre l'ultima settimana: inserisci una riga sopra l'ultima settimana e copia le formule dalla riga precedente.</t>
+  </si>
+  <si>
+    <t>Fase 1 — Analisi del dominio</t>
+  </si>
+  <si>
+    <t>Con Manuel: analisi del dominio, 2 personas, Stakeholder Matrix e matrice di tracciabilità.</t>
+  </si>
+  <si>
+    <t>docs/fase-1-analisi-dominio.md</t>
+  </si>
+  <si>
+    <t>Fase 2 — Specifiche dei requisiti</t>
+  </si>
+  <si>
+    <t>Con Manuel: SRS Light con requisiti funzionali (MoSCoW), requisiti non funzionali e casi d'uso.</t>
+  </si>
+  <si>
+    <t>docs/fase-2-specifiche-requisiti.md</t>
+  </si>
+  <si>
+    <t>Fase 3 — Architettura e user flow</t>
+  </si>
+  <si>
+    <t>Con Manuel: casi d'uso in Mermaid, flusso delle schermate, architettura ad alto livello e diagrammi di sequenza.</t>
+  </si>
+  <si>
+    <t>docs/fase-3-architettura-user-flow.md</t>
   </si>
 </sst>
 </file>
@@ -294,74 +321,74 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="8" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="1" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="1" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="1" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="1" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="1" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="1" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="5" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="5" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="14" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="166" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="8" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="166" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="1" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="1" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="166" fontId="1" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="1" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="1" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="166" fontId="1" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="5" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="166" fontId="5" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -384,7 +411,7 @@
     </dxf>
     <dxf>
       <font>
-        <b/>
+        <b val="0"/>
         <i val="0"/>
         <strike val="0"/>
         <condense val="0"/>
@@ -394,18 +421,31 @@
         <u val="none"/>
         <vertAlign val="baseline"/>
         <sz val="10"/>
-        <color rgb="FFFFFFFF"/>
+        <color theme="1"/>
         <name val="Arial"/>
         <family val="2"/>
         <scheme val="none"/>
       </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor rgb="FF1B2428"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
+        <color theme="1"/>
+        <name val="Arial"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
       <font>
@@ -426,25 +466,6 @@
       </font>
       <numFmt numFmtId="164" formatCode="0.0"/>
       <alignment horizontal="center" vertical="top" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="10"/>
-        <color theme="1"/>
-        <name val="Arial"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
       <font>
@@ -502,11 +523,11 @@
         <family val="2"/>
         <scheme val="none"/>
       </font>
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
       <font>
-        <b val="0"/>
+        <b/>
         <i val="0"/>
         <strike val="0"/>
         <condense val="0"/>
@@ -516,12 +537,37 @@
         <u val="none"/>
         <vertAlign val="baseline"/>
         <sz val="10"/>
-        <color theme="1"/>
+        <color rgb="FFFFFFFF"/>
         <name val="Arial"/>
         <family val="2"/>
         <scheme val="none"/>
       </font>
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FF1B2428"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFBF8F3"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <color rgb="FFFFFFFF"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF1B2428"/>
+        </patternFill>
+      </fill>
     </dxf>
     <dxf>
       <border>
@@ -545,31 +591,12 @@
         </horizontal>
       </border>
     </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFBF8F3"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <color rgb="FFFFFFFF"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF1B2428"/>
-        </patternFill>
-      </fill>
-    </dxf>
   </dxfs>
   <tableStyles count="1" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16">
     <tableStyle name="Libretto" pivot="0" count="3" xr9:uid="{C360CF7A-F8D2-42F1-A33C-C792160E0D97}">
-      <tableStyleElement type="wholeTable" dxfId="9"/>
-      <tableStyleElement type="headerRow" dxfId="11"/>
-      <tableStyleElement type="firstRowStripe" dxfId="10"/>
+      <tableStyleElement type="wholeTable" dxfId="11"/>
+      <tableStyleElement type="headerRow" dxfId="10"/>
+      <tableStyleElement type="firstRowStripe" dxfId="9"/>
     </tableStyle>
   </tableStyles>
   <extLst>
@@ -584,8 +611,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{AE054583-A50F-4EF9-8D40-13935D8BB6E2}" name="Registro" displayName="Registro" ref="A8:E10" totalsRowShown="0" headerRowDxfId="2" dataDxfId="8">
-  <autoFilter ref="A8:E10" xr:uid="{AE054583-A50F-4EF9-8D40-13935D8BB6E2}">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{AE054583-A50F-4EF9-8D40-13935D8BB6E2}" name="Registro" displayName="Registro" ref="A8:E13" totalsRowShown="0" headerRowDxfId="8" dataDxfId="7">
+  <autoFilter ref="A8:E13" xr:uid="{AE054583-A50F-4EF9-8D40-13935D8BB6E2}">
     <filterColumn colId="0" hiddenButton="1"/>
     <filterColumn colId="1" hiddenButton="1"/>
     <filterColumn colId="2" hiddenButton="1"/>
@@ -595,9 +622,9 @@
   <tableColumns count="5">
     <tableColumn id="1" xr3:uid="{48B5CA29-EC1B-4547-88A4-D993DC0EADC8}" name="Data" dataDxfId="6"/>
     <tableColumn id="2" xr3:uid="{420668F0-67D0-4D1C-B367-41B9FB7A2B44}" name="Attività" dataDxfId="5"/>
-    <tableColumn id="3" xr3:uid="{37736C0A-FA98-402A-B8D0-EC941A675BD3}" name="Ore" dataDxfId="3"/>
-    <tableColumn id="4" xr3:uid="{A0256299-8953-4BF5-9133-FC3A082528C4}" name="Descrizione" dataDxfId="4"/>
-    <tableColumn id="5" xr3:uid="{0ECB80BB-894B-49D0-96C5-62088A04A3D0}" name="Risultato / file" dataDxfId="7"/>
+    <tableColumn id="3" xr3:uid="{37736C0A-FA98-402A-B8D0-EC941A675BD3}" name="Ore" dataDxfId="4"/>
+    <tableColumn id="4" xr3:uid="{A0256299-8953-4BF5-9133-FC3A082528C4}" name="Descrizione" dataDxfId="3"/>
+    <tableColumn id="5" xr3:uid="{0ECB80BB-894B-49D0-96C5-62088A04A3D0}" name="Risultato / file" dataDxfId="2"/>
   </tableColumns>
   <tableStyleInfo name="Libretto" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -923,7 +950,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:E10"/>
+  <dimension ref="A1:E13"/>
   <sheetFormatPr defaultRowHeight="12.75" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="12.59765625" style="1" customWidth="1"/>
@@ -960,7 +987,7 @@
       </c>
       <c r="C5" s="7">
         <f>SUM(Registro[Ore])</f>
-        <v>0</v>
+        <v>3</v>
       </c>
     </row>
     <row r="6" spans="1:5" ht="13.15" x14ac:dyDescent="0.4">
@@ -973,58 +1000,109 @@
       </c>
     </row>
     <row r="7" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A7" s="10" t="s">
+      <c r="A7" s="31" t="s">
         <v>6</v>
       </c>
-      <c r="B7" s="9"/>
-      <c r="C7" s="9"/>
-      <c r="D7" s="9"/>
-      <c r="E7" s="9"/>
+      <c r="B7" s="32"/>
+      <c r="C7" s="32"/>
+      <c r="D7" s="32"/>
+      <c r="E7" s="32"/>
     </row>
     <row r="8" spans="1:5" ht="22.05" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A8" s="15" t="s">
+      <c r="A8" s="13" t="s">
         <v>7</v>
       </c>
-      <c r="B8" s="15" t="s">
+      <c r="B8" s="13" t="s">
         <v>8</v>
       </c>
-      <c r="C8" s="16" t="s">
+      <c r="C8" s="14" t="s">
         <v>9</v>
       </c>
-      <c r="D8" s="15" t="s">
+      <c r="D8" s="13" t="s">
         <v>10</v>
       </c>
-      <c r="E8" s="15" t="s">
+      <c r="E8" s="13" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="9" spans="1:5" ht="38.25" x14ac:dyDescent="0.35">
-      <c r="A9" s="13">
+      <c r="A9" s="11">
         <v>46294</v>
       </c>
-      <c r="B9" s="12" t="s">
+      <c r="B9" s="10" t="s">
         <v>12</v>
       </c>
-      <c r="C9" s="14"/>
-      <c r="D9" s="11" t="s">
+      <c r="C9" s="12"/>
+      <c r="D9" s="9" t="s">
         <v>13</v>
       </c>
-      <c r="E9" s="11" t="s">
+      <c r="E9" s="9" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="10" spans="1:5" ht="13.15" x14ac:dyDescent="0.35">
-      <c r="A10" s="13">
+    <row r="10" spans="1:5" ht="25.5" x14ac:dyDescent="0.35">
+      <c r="A10" s="11">
+        <v>46295</v>
+      </c>
+      <c r="B10" s="10" t="s">
+        <v>28</v>
+      </c>
+      <c r="C10" s="12">
+        <v>1</v>
+      </c>
+      <c r="D10" s="9" t="s">
+        <v>29</v>
+      </c>
+      <c r="E10" s="9" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" ht="25.5" x14ac:dyDescent="0.35">
+      <c r="A11" s="11">
+        <v>46295</v>
+      </c>
+      <c r="B11" s="10" t="s">
+        <v>31</v>
+      </c>
+      <c r="C11" s="12">
+        <v>1</v>
+      </c>
+      <c r="D11" s="9" t="s">
+        <v>32</v>
+      </c>
+      <c r="E11" s="9" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" ht="25.5" x14ac:dyDescent="0.35">
+      <c r="A12" s="11">
+        <v>46295</v>
+      </c>
+      <c r="B12" s="10" t="s">
+        <v>34</v>
+      </c>
+      <c r="C12" s="12">
+        <v>1</v>
+      </c>
+      <c r="D12" s="9" t="s">
+        <v>35</v>
+      </c>
+      <c r="E12" s="9" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" ht="13.15" x14ac:dyDescent="0.35">
+      <c r="A13" s="11">
         <v>46301</v>
       </c>
-      <c r="B10" s="12" t="s">
+      <c r="B13" s="10" t="s">
         <v>15</v>
       </c>
-      <c r="C10" s="14"/>
-      <c r="D10" s="11" t="s">
+      <c r="C13" s="12"/>
+      <c r="D13" s="9" t="s">
         <v>16</v>
       </c>
-      <c r="E10" s="11" t="s">
+      <c r="E13" s="9" t="s">
         <v>17</v>
       </c>
     </row>
@@ -1032,17 +1110,17 @@
   <mergeCells count="1">
     <mergeCell ref="A7:E7"/>
   </mergeCells>
-  <conditionalFormatting sqref="C9:C10">
+  <conditionalFormatting sqref="C9:C13">
     <cfRule type="expression" dxfId="1" priority="1" stopIfTrue="1">
       <formula>($B9&lt;&gt;"")*($C9="")</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="2">
-    <dataValidation type="date" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Data non valida" error="Scrivi la data come gg/mm/aaaa, per esempio 14/10/2026." sqref="A9:A10" xr:uid="{098F0742-FFAB-48A6-8604-D361C546CAF0}">
+    <dataValidation type="date" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Data non valida" error="Scrivi la data come gg/mm/aaaa, per esempio 14/10/2026." sqref="A9:A13" xr:uid="{098F0742-FFAB-48A6-8604-D361C546CAF0}">
       <formula1>46023</formula1>
       <formula2>47483</formula2>
     </dataValidation>
-    <dataValidation type="decimal" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Ore non valide" error="Scrivi le ore come numero tra 0 e 24 (1,5 = un'ora e mezza)." promptTitle="Ore dedicate" prompt="Numero di ore, anche decimale: 1,5 = un'ora e mezza." sqref="C9:C10" xr:uid="{14C505B7-43DA-4BD0-8687-D8FD2CC90D35}">
+    <dataValidation type="decimal" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Ore non valide" error="Scrivi le ore come numero tra 0 e 24 (1,5 = un'ora e mezza)." promptTitle="Ore dedicate" prompt="Numero di ore, anche decimale: 1,5 = un'ora e mezza." sqref="C9:C13" xr:uid="{14C505B7-43DA-4BD0-8687-D8FD2CC90D35}">
       <formula1>0</formula1>
       <formula2>24</formula2>
     </dataValidation>
@@ -1085,396 +1163,396 @@
       </c>
     </row>
     <row r="3" spans="1:5" ht="42" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A3" s="10" t="s">
+      <c r="A3" s="31" t="s">
         <v>19</v>
       </c>
-      <c r="B3" s="9"/>
-      <c r="C3" s="9"/>
-      <c r="D3" s="9"/>
-      <c r="E3" s="9"/>
+      <c r="B3" s="32"/>
+      <c r="C3" s="32"/>
+      <c r="D3" s="32"/>
+      <c r="E3" s="32"/>
     </row>
     <row r="5" spans="1:5" ht="22.05" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A5" s="18" t="s">
+      <c r="A5" s="16" t="s">
         <v>20</v>
       </c>
-      <c r="B5" s="18" t="s">
+      <c r="B5" s="16" t="s">
         <v>21</v>
       </c>
-      <c r="C5" s="18" t="s">
+      <c r="C5" s="16" t="s">
         <v>22</v>
       </c>
-      <c r="D5" s="18" t="s">
+      <c r="D5" s="16" t="s">
         <v>9</v>
       </c>
-      <c r="E5" s="18" t="s">
+      <c r="E5" s="16" t="s">
         <v>23</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A6" s="19">
+      <c r="A6" s="17">
         <v>46293</v>
       </c>
-      <c r="B6" s="20">
-        <f>A6+6</f>
+      <c r="B6" s="18">
+        <f t="shared" ref="B6:B21" si="0">A6+6</f>
         <v>46299</v>
       </c>
-      <c r="C6" s="21">
+      <c r="C6" s="19">
         <f>COUNTIFS(Registro[Data],"&gt;="&amp;A6,Registro[Data],"&lt;="&amp;B6)</f>
-        <v>1</v>
-      </c>
-      <c r="D6" s="22">
+        <v>4</v>
+      </c>
+      <c r="D6" s="20">
         <f>SUMIFS(Registro[Ore],Registro[Data],"&gt;="&amp;A6,Registro[Data],"&lt;="&amp;B6)</f>
-        <v>0</v>
-      </c>
-      <c r="E6" s="22">
+        <v>3</v>
+      </c>
+      <c r="E6" s="20">
         <f>SUM(D$6:D6)</f>
-        <v>0</v>
+        <v>3</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A7" s="23">
-        <f>A6+7</f>
+      <c r="A7" s="21">
+        <f t="shared" ref="A7:A21" si="1">A6+7</f>
         <v>46300</v>
       </c>
-      <c r="B7" s="23">
-        <f>A7+6</f>
+      <c r="B7" s="21">
+        <f t="shared" si="0"/>
         <v>46306</v>
       </c>
-      <c r="C7" s="24">
+      <c r="C7" s="22">
         <f>COUNTIFS(Registro[Data],"&gt;="&amp;A7,Registro[Data],"&lt;="&amp;B7)</f>
         <v>1</v>
       </c>
-      <c r="D7" s="25">
+      <c r="D7" s="23">
         <f>SUMIFS(Registro[Ore],Registro[Data],"&gt;="&amp;A7,Registro[Data],"&lt;="&amp;B7)</f>
         <v>0</v>
       </c>
-      <c r="E7" s="25">
+      <c r="E7" s="23">
         <f>SUM(D$6:D7)</f>
-        <v>0</v>
+        <v>3</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A8" s="20">
-        <f>A7+7</f>
+      <c r="A8" s="18">
+        <f t="shared" si="1"/>
         <v>46307</v>
       </c>
-      <c r="B8" s="20">
-        <f>A8+6</f>
+      <c r="B8" s="18">
+        <f t="shared" si="0"/>
         <v>46313</v>
       </c>
-      <c r="C8" s="21">
+      <c r="C8" s="19">
         <f>COUNTIFS(Registro[Data],"&gt;="&amp;A8,Registro[Data],"&lt;="&amp;B8)</f>
         <v>0</v>
       </c>
-      <c r="D8" s="22">
+      <c r="D8" s="20">
         <f>SUMIFS(Registro[Ore],Registro[Data],"&gt;="&amp;A8,Registro[Data],"&lt;="&amp;B8)</f>
         <v>0</v>
       </c>
-      <c r="E8" s="22">
+      <c r="E8" s="20">
         <f>SUM(D$6:D8)</f>
-        <v>0</v>
+        <v>3</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A9" s="23">
-        <f>A8+7</f>
+      <c r="A9" s="21">
+        <f t="shared" si="1"/>
         <v>46314</v>
       </c>
-      <c r="B9" s="23">
-        <f>A9+6</f>
+      <c r="B9" s="21">
+        <f t="shared" si="0"/>
         <v>46320</v>
       </c>
-      <c r="C9" s="24">
+      <c r="C9" s="22">
         <f>COUNTIFS(Registro[Data],"&gt;="&amp;A9,Registro[Data],"&lt;="&amp;B9)</f>
         <v>0</v>
       </c>
-      <c r="D9" s="25">
+      <c r="D9" s="23">
         <f>SUMIFS(Registro[Ore],Registro[Data],"&gt;="&amp;A9,Registro[Data],"&lt;="&amp;B9)</f>
         <v>0</v>
       </c>
-      <c r="E9" s="25">
+      <c r="E9" s="23">
         <f>SUM(D$6:D9)</f>
-        <v>0</v>
+        <v>3</v>
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A10" s="20">
-        <f>A9+7</f>
+      <c r="A10" s="18">
+        <f t="shared" si="1"/>
         <v>46321</v>
       </c>
-      <c r="B10" s="20">
-        <f>A10+6</f>
+      <c r="B10" s="18">
+        <f t="shared" si="0"/>
         <v>46327</v>
       </c>
-      <c r="C10" s="21">
+      <c r="C10" s="19">
         <f>COUNTIFS(Registro[Data],"&gt;="&amp;A10,Registro[Data],"&lt;="&amp;B10)</f>
         <v>0</v>
       </c>
-      <c r="D10" s="22">
+      <c r="D10" s="20">
         <f>SUMIFS(Registro[Ore],Registro[Data],"&gt;="&amp;A10,Registro[Data],"&lt;="&amp;B10)</f>
         <v>0</v>
       </c>
-      <c r="E10" s="22">
+      <c r="E10" s="20">
         <f>SUM(D$6:D10)</f>
-        <v>0</v>
+        <v>3</v>
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A11" s="23">
-        <f>A10+7</f>
+      <c r="A11" s="21">
+        <f t="shared" si="1"/>
         <v>46328</v>
       </c>
-      <c r="B11" s="23">
-        <f>A11+6</f>
+      <c r="B11" s="21">
+        <f t="shared" si="0"/>
         <v>46334</v>
       </c>
-      <c r="C11" s="24">
+      <c r="C11" s="22">
         <f>COUNTIFS(Registro[Data],"&gt;="&amp;A11,Registro[Data],"&lt;="&amp;B11)</f>
         <v>0</v>
       </c>
-      <c r="D11" s="25">
+      <c r="D11" s="23">
         <f>SUMIFS(Registro[Ore],Registro[Data],"&gt;="&amp;A11,Registro[Data],"&lt;="&amp;B11)</f>
         <v>0</v>
       </c>
-      <c r="E11" s="25">
+      <c r="E11" s="23">
         <f>SUM(D$6:D11)</f>
-        <v>0</v>
+        <v>3</v>
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A12" s="20">
-        <f>A11+7</f>
+      <c r="A12" s="18">
+        <f t="shared" si="1"/>
         <v>46335</v>
       </c>
-      <c r="B12" s="20">
-        <f>A12+6</f>
+      <c r="B12" s="18">
+        <f t="shared" si="0"/>
         <v>46341</v>
       </c>
-      <c r="C12" s="21">
+      <c r="C12" s="19">
         <f>COUNTIFS(Registro[Data],"&gt;="&amp;A12,Registro[Data],"&lt;="&amp;B12)</f>
         <v>0</v>
       </c>
-      <c r="D12" s="22">
+      <c r="D12" s="20">
         <f>SUMIFS(Registro[Ore],Registro[Data],"&gt;="&amp;A12,Registro[Data],"&lt;="&amp;B12)</f>
         <v>0</v>
       </c>
-      <c r="E12" s="22">
+      <c r="E12" s="20">
         <f>SUM(D$6:D12)</f>
-        <v>0</v>
+        <v>3</v>
       </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A13" s="23">
-        <f>A12+7</f>
+      <c r="A13" s="21">
+        <f t="shared" si="1"/>
         <v>46342</v>
       </c>
-      <c r="B13" s="23">
-        <f>A13+6</f>
+      <c r="B13" s="21">
+        <f t="shared" si="0"/>
         <v>46348</v>
       </c>
-      <c r="C13" s="24">
+      <c r="C13" s="22">
         <f>COUNTIFS(Registro[Data],"&gt;="&amp;A13,Registro[Data],"&lt;="&amp;B13)</f>
         <v>0</v>
       </c>
-      <c r="D13" s="25">
+      <c r="D13" s="23">
         <f>SUMIFS(Registro[Ore],Registro[Data],"&gt;="&amp;A13,Registro[Data],"&lt;="&amp;B13)</f>
         <v>0</v>
       </c>
-      <c r="E13" s="25">
+      <c r="E13" s="23">
         <f>SUM(D$6:D13)</f>
-        <v>0</v>
+        <v>3</v>
       </c>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A14" s="20">
-        <f>A13+7</f>
+      <c r="A14" s="18">
+        <f t="shared" si="1"/>
         <v>46349</v>
       </c>
-      <c r="B14" s="20">
-        <f>A14+6</f>
+      <c r="B14" s="18">
+        <f t="shared" si="0"/>
         <v>46355</v>
       </c>
-      <c r="C14" s="21">
+      <c r="C14" s="19">
         <f>COUNTIFS(Registro[Data],"&gt;="&amp;A14,Registro[Data],"&lt;="&amp;B14)</f>
         <v>0</v>
       </c>
-      <c r="D14" s="22">
+      <c r="D14" s="20">
         <f>SUMIFS(Registro[Ore],Registro[Data],"&gt;="&amp;A14,Registro[Data],"&lt;="&amp;B14)</f>
         <v>0</v>
       </c>
-      <c r="E14" s="22">
+      <c r="E14" s="20">
         <f>SUM(D$6:D14)</f>
-        <v>0</v>
+        <v>3</v>
       </c>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A15" s="23">
-        <f>A14+7</f>
+      <c r="A15" s="21">
+        <f t="shared" si="1"/>
         <v>46356</v>
       </c>
-      <c r="B15" s="23">
-        <f>A15+6</f>
+      <c r="B15" s="21">
+        <f t="shared" si="0"/>
         <v>46362</v>
       </c>
-      <c r="C15" s="24">
+      <c r="C15" s="22">
         <f>COUNTIFS(Registro[Data],"&gt;="&amp;A15,Registro[Data],"&lt;="&amp;B15)</f>
         <v>0</v>
       </c>
-      <c r="D15" s="25">
+      <c r="D15" s="23">
         <f>SUMIFS(Registro[Ore],Registro[Data],"&gt;="&amp;A15,Registro[Data],"&lt;="&amp;B15)</f>
         <v>0</v>
       </c>
-      <c r="E15" s="25">
+      <c r="E15" s="23">
         <f>SUM(D$6:D15)</f>
-        <v>0</v>
+        <v>3</v>
       </c>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A16" s="20">
-        <f>A15+7</f>
+      <c r="A16" s="18">
+        <f t="shared" si="1"/>
         <v>46363</v>
       </c>
-      <c r="B16" s="20">
-        <f>A16+6</f>
+      <c r="B16" s="18">
+        <f t="shared" si="0"/>
         <v>46369</v>
       </c>
-      <c r="C16" s="21">
+      <c r="C16" s="19">
         <f>COUNTIFS(Registro[Data],"&gt;="&amp;A16,Registro[Data],"&lt;="&amp;B16)</f>
         <v>0</v>
       </c>
-      <c r="D16" s="22">
+      <c r="D16" s="20">
         <f>SUMIFS(Registro[Ore],Registro[Data],"&gt;="&amp;A16,Registro[Data],"&lt;="&amp;B16)</f>
         <v>0</v>
       </c>
-      <c r="E16" s="22">
+      <c r="E16" s="20">
         <f>SUM(D$6:D16)</f>
-        <v>0</v>
+        <v>3</v>
       </c>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A17" s="23">
-        <f>A16+7</f>
+      <c r="A17" s="21">
+        <f t="shared" si="1"/>
         <v>46370</v>
       </c>
-      <c r="B17" s="23">
-        <f>A17+6</f>
+      <c r="B17" s="21">
+        <f t="shared" si="0"/>
         <v>46376</v>
       </c>
-      <c r="C17" s="24">
+      <c r="C17" s="22">
         <f>COUNTIFS(Registro[Data],"&gt;="&amp;A17,Registro[Data],"&lt;="&amp;B17)</f>
         <v>0</v>
       </c>
-      <c r="D17" s="25">
+      <c r="D17" s="23">
         <f>SUMIFS(Registro[Ore],Registro[Data],"&gt;="&amp;A17,Registro[Data],"&lt;="&amp;B17)</f>
         <v>0</v>
       </c>
-      <c r="E17" s="25">
+      <c r="E17" s="23">
         <f>SUM(D$6:D17)</f>
-        <v>0</v>
+        <v>3</v>
       </c>
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A18" s="20">
-        <f>A17+7</f>
+      <c r="A18" s="18">
+        <f t="shared" si="1"/>
         <v>46377</v>
       </c>
-      <c r="B18" s="20">
-        <f>A18+6</f>
+      <c r="B18" s="18">
+        <f t="shared" si="0"/>
         <v>46383</v>
       </c>
-      <c r="C18" s="21">
+      <c r="C18" s="19">
         <f>COUNTIFS(Registro[Data],"&gt;="&amp;A18,Registro[Data],"&lt;="&amp;B18)</f>
         <v>0</v>
       </c>
-      <c r="D18" s="22">
+      <c r="D18" s="20">
         <f>SUMIFS(Registro[Ore],Registro[Data],"&gt;="&amp;A18,Registro[Data],"&lt;="&amp;B18)</f>
         <v>0</v>
       </c>
-      <c r="E18" s="22">
+      <c r="E18" s="20">
         <f>SUM(D$6:D18)</f>
-        <v>0</v>
+        <v>3</v>
       </c>
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A19" s="23">
-        <f>A18+7</f>
+      <c r="A19" s="21">
+        <f t="shared" si="1"/>
         <v>46384</v>
       </c>
-      <c r="B19" s="23">
-        <f>A19+6</f>
+      <c r="B19" s="21">
+        <f t="shared" si="0"/>
         <v>46390</v>
       </c>
-      <c r="C19" s="24">
+      <c r="C19" s="22">
         <f>COUNTIFS(Registro[Data],"&gt;="&amp;A19,Registro[Data],"&lt;="&amp;B19)</f>
         <v>0</v>
       </c>
-      <c r="D19" s="25">
+      <c r="D19" s="23">
         <f>SUMIFS(Registro[Ore],Registro[Data],"&gt;="&amp;A19,Registro[Data],"&lt;="&amp;B19)</f>
         <v>0</v>
       </c>
-      <c r="E19" s="25">
+      <c r="E19" s="23">
         <f>SUM(D$6:D19)</f>
-        <v>0</v>
+        <v>3</v>
       </c>
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A20" s="20">
-        <f>A19+7</f>
+      <c r="A20" s="18">
+        <f t="shared" si="1"/>
         <v>46391</v>
       </c>
-      <c r="B20" s="20">
-        <f>A20+6</f>
+      <c r="B20" s="18">
+        <f t="shared" si="0"/>
         <v>46397</v>
       </c>
-      <c r="C20" s="21">
+      <c r="C20" s="19">
         <f>COUNTIFS(Registro[Data],"&gt;="&amp;A20,Registro[Data],"&lt;="&amp;B20)</f>
         <v>0</v>
       </c>
-      <c r="D20" s="22">
+      <c r="D20" s="20">
         <f>SUMIFS(Registro[Ore],Registro[Data],"&gt;="&amp;A20,Registro[Data],"&lt;="&amp;B20)</f>
         <v>0</v>
       </c>
-      <c r="E20" s="22">
+      <c r="E20" s="20">
         <f>SUM(D$6:D20)</f>
-        <v>0</v>
+        <v>3</v>
       </c>
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A21" s="26">
-        <f>A20+7</f>
+      <c r="A21" s="24">
+        <f t="shared" si="1"/>
         <v>46398</v>
       </c>
-      <c r="B21" s="26">
-        <f>A21+6</f>
+      <c r="B21" s="24">
+        <f t="shared" si="0"/>
         <v>46404</v>
       </c>
-      <c r="C21" s="27">
+      <c r="C21" s="25">
         <f>COUNTIFS(Registro[Data],"&gt;="&amp;A21,Registro[Data],"&lt;="&amp;B21)</f>
         <v>0</v>
       </c>
-      <c r="D21" s="28">
+      <c r="D21" s="26">
         <f>SUMIFS(Registro[Ore],Registro[Data],"&gt;="&amp;A21,Registro[Data],"&lt;="&amp;B21)</f>
         <v>0</v>
       </c>
-      <c r="E21" s="28">
+      <c r="E21" s="26">
         <f>SUM(D$6:D21)</f>
-        <v>0</v>
+        <v>3</v>
       </c>
     </row>
     <row r="22" spans="1:5" ht="13.15" x14ac:dyDescent="0.4">
-      <c r="A22" s="29" t="s">
+      <c r="A22" s="27" t="s">
         <v>24</v>
       </c>
-      <c r="B22" s="30"/>
-      <c r="C22" s="31">
+      <c r="B22" s="28"/>
+      <c r="C22" s="29">
         <f>SUM(C6:C21)</f>
-        <v>2</v>
-      </c>
-      <c r="D22" s="32">
+        <v>5</v>
+      </c>
+      <c r="D22" s="30">
         <f>SUM(D6:D21)</f>
-        <v>0</v>
-      </c>
-      <c r="E22" s="30"/>
+        <v>3</v>
+      </c>
+      <c r="E22" s="28"/>
     </row>
     <row r="24" spans="1:5" ht="13.15" x14ac:dyDescent="0.4">
       <c r="A24" s="6" t="s">
@@ -1482,9 +1560,9 @@
       </c>
       <c r="B24" s="6"/>
       <c r="C24" s="6"/>
-      <c r="D24" s="17">
+      <c r="D24" s="15">
         <f>SUM(Registro[Ore])</f>
-        <v>0</v>
+        <v>3</v>
       </c>
     </row>
     <row r="25" spans="1:5" ht="13.15" x14ac:dyDescent="0.4">
@@ -1493,19 +1571,19 @@
       </c>
       <c r="B25" s="6"/>
       <c r="C25" s="6"/>
-      <c r="D25" s="17">
+      <c r="D25" s="15">
         <f>D24-D22</f>
         <v>0</v>
       </c>
     </row>
     <row r="26" spans="1:5" ht="42" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A26" s="10" t="s">
+      <c r="A26" s="31" t="s">
         <v>27</v>
       </c>
-      <c r="B26" s="9"/>
-      <c r="C26" s="9"/>
-      <c r="D26" s="9"/>
-      <c r="E26" s="9"/>
+      <c r="B26" s="32"/>
+      <c r="C26" s="32"/>
+      <c r="D26" s="32"/>
+      <c r="E26" s="32"/>
     </row>
   </sheetData>
   <mergeCells count="2">

</xml_diff>

<commit_message>
Libretti: 2,5 ore ciascuna per le Fasi 2 e 3
Le Fasi 2 e 3 sono state scritte insieme da Manuel e Marco: stima di
2,5 ore per ogni fase in entrambi i libretti.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/libretti/marco-buffa.xlsx
+++ b/docs/libretti/marco-buffa.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\bulla\Documents\Ing-software-v1\docs\libretti\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{18DB9327-8DE3-46DC-9CA1-1444C9B38741}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C48C8B71-EAEF-4D4F-AB1B-9708293CFCA3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" xr2:uid="{69E2A5B4-4109-48EA-BF49-3C21B144A51A}"/>
   </bookViews>
@@ -987,7 +987,7 @@
       </c>
       <c r="C5" s="7">
         <f>SUM(Registro[Ore])</f>
-        <v>3</v>
+        <v>6</v>
       </c>
     </row>
     <row r="6" spans="1:5" ht="13.15" x14ac:dyDescent="0.4">
@@ -1065,7 +1065,7 @@
         <v>31</v>
       </c>
       <c r="C11" s="12">
-        <v>1</v>
+        <v>2.5</v>
       </c>
       <c r="D11" s="9" t="s">
         <v>32</v>
@@ -1082,7 +1082,7 @@
         <v>34</v>
       </c>
       <c r="C12" s="12">
-        <v>1</v>
+        <v>2.5</v>
       </c>
       <c r="D12" s="9" t="s">
         <v>35</v>
@@ -1202,11 +1202,11 @@
       </c>
       <c r="D6" s="20">
         <f>SUMIFS(Registro[Ore],Registro[Data],"&gt;="&amp;A6,Registro[Data],"&lt;="&amp;B6)</f>
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="E6" s="20">
         <f>SUM(D$6:D6)</f>
-        <v>3</v>
+        <v>6</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.35">
@@ -1228,7 +1228,7 @@
       </c>
       <c r="E7" s="23">
         <f>SUM(D$6:D7)</f>
-        <v>3</v>
+        <v>6</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.35">
@@ -1250,7 +1250,7 @@
       </c>
       <c r="E8" s="20">
         <f>SUM(D$6:D8)</f>
-        <v>3</v>
+        <v>6</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.35">
@@ -1272,7 +1272,7 @@
       </c>
       <c r="E9" s="23">
         <f>SUM(D$6:D9)</f>
-        <v>3</v>
+        <v>6</v>
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.35">
@@ -1294,7 +1294,7 @@
       </c>
       <c r="E10" s="20">
         <f>SUM(D$6:D10)</f>
-        <v>3</v>
+        <v>6</v>
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.35">
@@ -1316,7 +1316,7 @@
       </c>
       <c r="E11" s="23">
         <f>SUM(D$6:D11)</f>
-        <v>3</v>
+        <v>6</v>
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.35">
@@ -1338,7 +1338,7 @@
       </c>
       <c r="E12" s="20">
         <f>SUM(D$6:D12)</f>
-        <v>3</v>
+        <v>6</v>
       </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.35">
@@ -1360,7 +1360,7 @@
       </c>
       <c r="E13" s="23">
         <f>SUM(D$6:D13)</f>
-        <v>3</v>
+        <v>6</v>
       </c>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.35">
@@ -1382,7 +1382,7 @@
       </c>
       <c r="E14" s="20">
         <f>SUM(D$6:D14)</f>
-        <v>3</v>
+        <v>6</v>
       </c>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.35">
@@ -1404,7 +1404,7 @@
       </c>
       <c r="E15" s="23">
         <f>SUM(D$6:D15)</f>
-        <v>3</v>
+        <v>6</v>
       </c>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.35">
@@ -1426,7 +1426,7 @@
       </c>
       <c r="E16" s="20">
         <f>SUM(D$6:D16)</f>
-        <v>3</v>
+        <v>6</v>
       </c>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.35">
@@ -1448,7 +1448,7 @@
       </c>
       <c r="E17" s="23">
         <f>SUM(D$6:D17)</f>
-        <v>3</v>
+        <v>6</v>
       </c>
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.35">
@@ -1470,7 +1470,7 @@
       </c>
       <c r="E18" s="20">
         <f>SUM(D$6:D18)</f>
-        <v>3</v>
+        <v>6</v>
       </c>
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.35">
@@ -1492,7 +1492,7 @@
       </c>
       <c r="E19" s="23">
         <f>SUM(D$6:D19)</f>
-        <v>3</v>
+        <v>6</v>
       </c>
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.35">
@@ -1514,7 +1514,7 @@
       </c>
       <c r="E20" s="20">
         <f>SUM(D$6:D20)</f>
-        <v>3</v>
+        <v>6</v>
       </c>
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.35">
@@ -1536,7 +1536,7 @@
       </c>
       <c r="E21" s="26">
         <f>SUM(D$6:D21)</f>
-        <v>3</v>
+        <v>6</v>
       </c>
     </row>
     <row r="22" spans="1:5" ht="13.15" x14ac:dyDescent="0.4">
@@ -1550,7 +1550,7 @@
       </c>
       <c r="D22" s="30">
         <f>SUM(D6:D21)</f>
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="E22" s="28"/>
     </row>
@@ -1562,7 +1562,7 @@
       <c r="C24" s="6"/>
       <c r="D24" s="15">
         <f>SUM(Registro[Ore])</f>
-        <v>3</v>
+        <v>6</v>
       </c>
     </row>
     <row r="25" spans="1:5" ht="13.15" x14ac:dyDescent="0.4">

</xml_diff>

<commit_message>
Libretto Marco: modifiche alla mappa
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/libretti/marco-buffa.xlsx
+++ b/docs/libretti/marco-buffa.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\bulla\Documents\Ing-software-v1\docs\libretti\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C48C8B71-EAEF-4D4F-AB1B-9708293CFCA3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{53965E7F-489F-4C64-81A2-143D127F2243}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" xr2:uid="{69E2A5B4-4109-48EA-BF49-3C21B144A51A}"/>
   </bookViews>
@@ -43,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="39" uniqueCount="37">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="42" uniqueCount="40">
   <si>
     <t>Libretto delle attività</t>
   </si>
@@ -154,6 +154,15 @@
   </si>
   <si>
     <t>docs/fase-3-architettura-user-flow.md</t>
+  </si>
+  <si>
+    <t>Modifiche mappa</t>
+  </si>
+  <si>
+    <t>Trovato lo stile di mappa MapTiler senza negozi e bar e adattato lo sfondo del sito, con chiave in file locale e ripiego su OpenStreetMap.</t>
+  </si>
+  <si>
+    <t>versione-corrente/frontend/src/lib/sfondo.js, MappaLeaflet.jsx, Copertina.jsx</t>
   </si>
 </sst>
 </file>
@@ -611,8 +620,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{AE054583-A50F-4EF9-8D40-13935D8BB6E2}" name="Registro" displayName="Registro" ref="A8:E13" totalsRowShown="0" headerRowDxfId="8" dataDxfId="7">
-  <autoFilter ref="A8:E13" xr:uid="{AE054583-A50F-4EF9-8D40-13935D8BB6E2}">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{AE054583-A50F-4EF9-8D40-13935D8BB6E2}" name="Registro" displayName="Registro" ref="A8:E14" totalsRowShown="0" headerRowDxfId="8" dataDxfId="7">
+  <autoFilter ref="A8:E14" xr:uid="{AE054583-A50F-4EF9-8D40-13935D8BB6E2}">
     <filterColumn colId="0" hiddenButton="1"/>
     <filterColumn colId="1" hiddenButton="1"/>
     <filterColumn colId="2" hiddenButton="1"/>
@@ -950,7 +959,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:E13"/>
+  <dimension ref="A1:E14"/>
   <sheetFormatPr defaultRowHeight="12.75" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="12.59765625" style="1" customWidth="1"/>
@@ -987,7 +996,7 @@
       </c>
       <c r="C5" s="7">
         <f>SUM(Registro[Ore])</f>
-        <v>6</v>
+        <v>9</v>
       </c>
     </row>
     <row r="6" spans="1:5" ht="13.15" x14ac:dyDescent="0.4">
@@ -1106,21 +1115,38 @@
         <v>17</v>
       </c>
     </row>
+    <row r="14" spans="1:5" ht="25.5" x14ac:dyDescent="0.35">
+      <c r="A14" s="11">
+        <v>46309</v>
+      </c>
+      <c r="B14" s="10" t="s">
+        <v>37</v>
+      </c>
+      <c r="C14" s="12">
+        <v>3</v>
+      </c>
+      <c r="D14" s="9" t="s">
+        <v>38</v>
+      </c>
+      <c r="E14" s="9" t="s">
+        <v>39</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A7:E7"/>
   </mergeCells>
-  <conditionalFormatting sqref="C9:C13">
+  <conditionalFormatting sqref="C9:C14">
     <cfRule type="expression" dxfId="1" priority="1" stopIfTrue="1">
       <formula>($B9&lt;&gt;"")*($C9="")</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="2">
-    <dataValidation type="date" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Data non valida" error="Scrivi la data come gg/mm/aaaa, per esempio 14/10/2026." sqref="A9:A13" xr:uid="{098F0742-FFAB-48A6-8604-D361C546CAF0}">
+    <dataValidation type="date" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Data non valida" error="Scrivi la data come gg/mm/aaaa, per esempio 14/10/2026." sqref="A9:A14" xr:uid="{098F0742-FFAB-48A6-8604-D361C546CAF0}">
       <formula1>46023</formula1>
       <formula2>47483</formula2>
     </dataValidation>
-    <dataValidation type="decimal" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Ore non valide" error="Scrivi le ore come numero tra 0 e 24 (1,5 = un'ora e mezza)." promptTitle="Ore dedicate" prompt="Numero di ore, anche decimale: 1,5 = un'ora e mezza." sqref="C9:C13" xr:uid="{14C505B7-43DA-4BD0-8687-D8FD2CC90D35}">
+    <dataValidation type="decimal" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Ore non valide" error="Scrivi le ore come numero tra 0 e 24 (1,5 = un'ora e mezza)." promptTitle="Ore dedicate" prompt="Numero di ore, anche decimale: 1,5 = un'ora e mezza." sqref="C9:C14" xr:uid="{14C505B7-43DA-4BD0-8687-D8FD2CC90D35}">
       <formula1>0</formula1>
       <formula2>24</formula2>
     </dataValidation>
@@ -1242,15 +1268,15 @@
       </c>
       <c r="C8" s="19">
         <f>COUNTIFS(Registro[Data],"&gt;="&amp;A8,Registro[Data],"&lt;="&amp;B8)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D8" s="20">
         <f>SUMIFS(Registro[Ore],Registro[Data],"&gt;="&amp;A8,Registro[Data],"&lt;="&amp;B8)</f>
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="E8" s="20">
         <f>SUM(D$6:D8)</f>
-        <v>6</v>
+        <v>9</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.35">
@@ -1272,7 +1298,7 @@
       </c>
       <c r="E9" s="23">
         <f>SUM(D$6:D9)</f>
-        <v>6</v>
+        <v>9</v>
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.35">
@@ -1294,7 +1320,7 @@
       </c>
       <c r="E10" s="20">
         <f>SUM(D$6:D10)</f>
-        <v>6</v>
+        <v>9</v>
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.35">
@@ -1316,7 +1342,7 @@
       </c>
       <c r="E11" s="23">
         <f>SUM(D$6:D11)</f>
-        <v>6</v>
+        <v>9</v>
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.35">
@@ -1338,7 +1364,7 @@
       </c>
       <c r="E12" s="20">
         <f>SUM(D$6:D12)</f>
-        <v>6</v>
+        <v>9</v>
       </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.35">
@@ -1360,7 +1386,7 @@
       </c>
       <c r="E13" s="23">
         <f>SUM(D$6:D13)</f>
-        <v>6</v>
+        <v>9</v>
       </c>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.35">
@@ -1382,7 +1408,7 @@
       </c>
       <c r="E14" s="20">
         <f>SUM(D$6:D14)</f>
-        <v>6</v>
+        <v>9</v>
       </c>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.35">
@@ -1404,7 +1430,7 @@
       </c>
       <c r="E15" s="23">
         <f>SUM(D$6:D15)</f>
-        <v>6</v>
+        <v>9</v>
       </c>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.35">
@@ -1426,7 +1452,7 @@
       </c>
       <c r="E16" s="20">
         <f>SUM(D$6:D16)</f>
-        <v>6</v>
+        <v>9</v>
       </c>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.35">
@@ -1448,7 +1474,7 @@
       </c>
       <c r="E17" s="23">
         <f>SUM(D$6:D17)</f>
-        <v>6</v>
+        <v>9</v>
       </c>
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.35">
@@ -1470,7 +1496,7 @@
       </c>
       <c r="E18" s="20">
         <f>SUM(D$6:D18)</f>
-        <v>6</v>
+        <v>9</v>
       </c>
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.35">
@@ -1492,7 +1518,7 @@
       </c>
       <c r="E19" s="23">
         <f>SUM(D$6:D19)</f>
-        <v>6</v>
+        <v>9</v>
       </c>
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.35">
@@ -1514,7 +1540,7 @@
       </c>
       <c r="E20" s="20">
         <f>SUM(D$6:D20)</f>
-        <v>6</v>
+        <v>9</v>
       </c>
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.35">
@@ -1536,7 +1562,7 @@
       </c>
       <c r="E21" s="26">
         <f>SUM(D$6:D21)</f>
-        <v>6</v>
+        <v>9</v>
       </c>
     </row>
     <row r="22" spans="1:5" ht="13.15" x14ac:dyDescent="0.4">
@@ -1546,11 +1572,11 @@
       <c r="B22" s="28"/>
       <c r="C22" s="29">
         <f>SUM(C6:C21)</f>
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D22" s="30">
         <f>SUM(D6:D21)</f>
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="E22" s="28"/>
     </row>
@@ -1562,7 +1588,7 @@
       <c r="C24" s="6"/>
       <c r="D24" s="15">
         <f>SUM(Registro[Ore])</f>
-        <v>6</v>
+        <v>9</v>
       </c>
     </row>
     <row r="25" spans="1:5" ht="13.15" x14ac:dyDescent="0.4">

</xml_diff>